<commit_message>
docs(survey): pin the workbook's evidence in a tracked receipt
The workbook cited raw manifests under tmp/, which is not tracked: cleaning the
scratch directory would have left every row pointing at a file that no longer
exists. This adds `data/workbook_runs_20261025.json` as the single source the
workbook reads, and the workbook's `evidence` column now names a key in it.

The receipt keeps the audit fields (selection, resources, test_results,
protocol identity) and drops `candidate_runs`, the per-epoch validation trace
that is 40% of a manifest's bytes, recording its SHA-256 instead. The
clean-support `split_ref` is hoisted once and keyed by digest: nine runs shared
one 65 KB membership list. 5.6 MB of manifests becomes an 819 KB receipt, and
each entry still names its original path, byte size and manifest SHA-256.

Rebuilding the workbook no longer needs the raw manifests at all.
</commit_message>
<xml_diff>
--- a/docs/research/pu_survey/data/PU_Survey_results_20261025.xlsx
+++ b/docs/research/pu_survey/data/PU_Survey_results_20261025.xlsx
@@ -659,7 +659,7 @@
       </c>
       <c r="AH1" s="1" t="inlineStr">
         <is>
-          <t>evidence_manifest</t>
+          <t>evidence</t>
         </is>
       </c>
       <c r="AI1" s="1" t="inlineStr">
@@ -802,7 +802,7 @@
       </c>
       <c r="AH2" t="inlineStr">
         <is>
-          <t>tmp/wb_cifar_20261025/holistic_pu_c0.1/manifest.json</t>
+          <t>docs/research/pu_survey/data/workbook_runs_20261025.json#w-cifar-adapter/holistic_pu/cifar10/c0.1/seed0</t>
         </is>
       </c>
       <c r="AI2" t="inlineStr">
@@ -945,7 +945,7 @@
       </c>
       <c r="AH3" t="inlineStr">
         <is>
-          <t>tmp/wb_cifar_20261025/holistic_pu_c0.3/manifest.json</t>
+          <t>docs/research/pu_survey/data/workbook_runs_20261025.json#w-cifar-adapter/holistic_pu/cifar10/c0.3/seed0</t>
         </is>
       </c>
       <c r="AI3" t="inlineStr">
@@ -1088,7 +1088,7 @@
       </c>
       <c r="AH4" t="inlineStr">
         <is>
-          <t>tmp/wb_cifar_20261025/holistic_pu_c0.5/manifest.json</t>
+          <t>docs/research/pu_survey/data/workbook_runs_20261025.json#w-cifar-adapter/holistic_pu/cifar10/c0.5/seed0</t>
         </is>
       </c>
       <c r="AI4" t="inlineStr">
@@ -1231,7 +1231,7 @@
       </c>
       <c r="AH5" t="inlineStr">
         <is>
-          <t>tmp/wb_cifar_20261025/robust_pu_c0.1/manifest.json</t>
+          <t>docs/research/pu_survey/data/workbook_runs_20261025.json#w-cifar-adapter/robust_pu/cifar10/c0.1/seed0</t>
         </is>
       </c>
       <c r="AI5" t="inlineStr">
@@ -1374,7 +1374,7 @@
       </c>
       <c r="AH6" t="inlineStr">
         <is>
-          <t>tmp/wb_cifar_20261025/robust_pu_c0.3/manifest.json</t>
+          <t>docs/research/pu_survey/data/workbook_runs_20261025.json#w-cifar-adapter/robust_pu/cifar10/c0.3/seed0</t>
         </is>
       </c>
       <c r="AI6" t="inlineStr">
@@ -1517,7 +1517,7 @@
       </c>
       <c r="AH7" t="inlineStr">
         <is>
-          <t>tmp/wb_cifar_20261025/robust_pu_c0.5/manifest.json</t>
+          <t>docs/research/pu_survey/data/workbook_runs_20261025.json#w-cifar-adapter/robust_pu/cifar10/c0.5/seed0</t>
         </is>
       </c>
       <c r="AI7" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="AH8" t="inlineStr">
         <is>
-          <t>tmp/wb_cifar_20261025/split_pu_c0.1/manifest.json</t>
+          <t>docs/research/pu_survey/data/workbook_runs_20261025.json#w-cifar-adapter/split_pu/cifar10/c0.1/seed0</t>
         </is>
       </c>
       <c r="AI8" t="inlineStr">
@@ -1803,7 +1803,7 @@
       </c>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>tmp/wb_cifar_20261025/split_pu_c0.3/manifest.json</t>
+          <t>docs/research/pu_survey/data/workbook_runs_20261025.json#w-cifar-adapter/split_pu/cifar10/c0.3/seed0</t>
         </is>
       </c>
       <c r="AI9" t="inlineStr">
@@ -1946,7 +1946,7 @@
       </c>
       <c r="AH10" t="inlineStr">
         <is>
-          <t>tmp/wb_cifar_20261025/split_pu_c0.5/manifest.json</t>
+          <t>docs/research/pu_survey/data/workbook_runs_20261025.json#w-cifar-adapter/split_pu/cifar10/c0.5/seed0</t>
         </is>
       </c>
       <c r="AI10" t="inlineStr">
@@ -2084,7 +2084,7 @@
       </c>
       <c r="AH11" t="inlineStr">
         <is>
-          <t>docs/research/pu_survey/data/survey_recipe_formal_run_20261025.json</t>
+          <t>docs/research/pu_survey/data/workbook_runs_20261025.json#w-genpu-formal/genpu/cifar10/c0.5/seed0</t>
         </is>
       </c>
       <c r="AI11" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="AH12" t="inlineStr">
         <is>
-          <t>tmp/wb_20261025/holistic_pu_c0.1/os/c_0.1/seed_0/manifest.json</t>
+          <t>docs/research/pu_survey/data/workbook_runs_20261025.json#w-spambase-grid/holistic_pu/spambase/c0.1/seed0</t>
         </is>
       </c>
       <c r="AI12" t="inlineStr">
@@ -2364,7 +2364,7 @@
       </c>
       <c r="AH13" t="inlineStr">
         <is>
-          <t>tmp/wb_20261025/holistic_pu_c0.3/os/c_0.3/seed_0/manifest.json</t>
+          <t>docs/research/pu_survey/data/workbook_runs_20261025.json#w-spambase-grid/holistic_pu/spambase/c0.3/seed0</t>
         </is>
       </c>
       <c r="AI13" t="inlineStr">
@@ -2504,7 +2504,7 @@
       </c>
       <c r="AH14" t="inlineStr">
         <is>
-          <t>tmp/wb_20261025/holistic_pu_c0.5/os/c_0.5/seed_0/manifest.json</t>
+          <t>docs/research/pu_survey/data/workbook_runs_20261025.json#w-spambase-grid/holistic_pu/spambase/c0.5/seed0</t>
         </is>
       </c>
       <c r="AI14" t="inlineStr">
@@ -2644,7 +2644,7 @@
       </c>
       <c r="AH15" t="inlineStr">
         <is>
-          <t>tmp/wb_20261025/lagam_c0.1/os/c_0.1/seed_0/manifest.json</t>
+          <t>docs/research/pu_survey/data/workbook_runs_20261025.json#w-spambase-grid/lagam/spambase/c0.1/seed0</t>
         </is>
       </c>
       <c r="AI15" t="inlineStr">
@@ -2784,7 +2784,7 @@
       </c>
       <c r="AH16" t="inlineStr">
         <is>
-          <t>tmp/wb_20261025/lagam_c0.3/os/c_0.3/seed_0/manifest.json</t>
+          <t>docs/research/pu_survey/data/workbook_runs_20261025.json#w-spambase-grid/lagam/spambase/c0.3/seed0</t>
         </is>
       </c>
       <c r="AI16" t="inlineStr">
@@ -2924,7 +2924,7 @@
       </c>
       <c r="AH17" t="inlineStr">
         <is>
-          <t>tmp/wb_20261025/lagam_c0.5/os/c_0.5/seed_0/manifest.json</t>
+          <t>docs/research/pu_survey/data/workbook_runs_20261025.json#w-spambase-grid/lagam/spambase/c0.5/seed0</t>
         </is>
       </c>
       <c r="AI17" t="inlineStr">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="AH18" t="inlineStr">
         <is>
-          <t>tmp/wb_20261025/pulns_c0.1/os/c_0.1/seed_0/manifest.json</t>
+          <t>docs/research/pu_survey/data/workbook_runs_20261025.json#w-spambase-grid/pulns/spambase/c0.1/seed0</t>
         </is>
       </c>
       <c r="AI18" t="inlineStr">
@@ -3204,7 +3204,7 @@
       </c>
       <c r="AH19" t="inlineStr">
         <is>
-          <t>tmp/wb_20261025/pulns_c0.3/os/c_0.3/seed_0/manifest.json</t>
+          <t>docs/research/pu_survey/data/workbook_runs_20261025.json#w-spambase-grid/pulns/spambase/c0.3/seed0</t>
         </is>
       </c>
       <c r="AI19" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="AH20" t="inlineStr">
         <is>
-          <t>tmp/wb_20261025/pulns_c0.5/os/c_0.5/seed_0/manifest.json</t>
+          <t>docs/research/pu_survey/data/workbook_runs_20261025.json#w-spambase-grid/pulns/spambase/c0.5/seed0</t>
         </is>
       </c>
       <c r="AI20" t="inlineStr">
@@ -3484,7 +3484,7 @@
       </c>
       <c r="AH21" t="inlineStr">
         <is>
-          <t>tmp/wb_20261025/robust_pu_c0.1/ts/c_0.1/seed_0/manifest.json</t>
+          <t>docs/research/pu_survey/data/workbook_runs_20261025.json#w-spambase-grid/robust_pu/spambase/c0.1/seed0</t>
         </is>
       </c>
       <c r="AI21" t="inlineStr">
@@ -3624,7 +3624,7 @@
       </c>
       <c r="AH22" t="inlineStr">
         <is>
-          <t>tmp/wb_20261025/robust_pu_c0.3/ts/c_0.3/seed_0/manifest.json</t>
+          <t>docs/research/pu_survey/data/workbook_runs_20261025.json#w-spambase-grid/robust_pu/spambase/c0.3/seed0</t>
         </is>
       </c>
       <c r="AI22" t="inlineStr">
@@ -3764,7 +3764,7 @@
       </c>
       <c r="AH23" t="inlineStr">
         <is>
-          <t>tmp/wb_20261025/robust_pu_c0.5/ts/c_0.5/seed_0/manifest.json</t>
+          <t>docs/research/pu_survey/data/workbook_runs_20261025.json#w-spambase-grid/robust_pu/spambase/c0.5/seed0</t>
         </is>
       </c>
       <c r="AI23" t="inlineStr">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="AH24" t="inlineStr">
         <is>
-          <t>tmp/wb_20261025/self_pu_full_meta_c0.1/ts/c_0.1/seed_0/manifest.json</t>
+          <t>docs/research/pu_survey/data/workbook_runs_20261025.json#w-spambase-grid/self_pu_full_meta/spambase/c0.1/seed0</t>
         </is>
       </c>
       <c r="AI24" t="inlineStr">
@@ -4044,7 +4044,7 @@
       </c>
       <c r="AH25" t="inlineStr">
         <is>
-          <t>tmp/wb_20261025/self_pu_full_meta_c0.3/ts/c_0.3/seed_0/manifest.json</t>
+          <t>docs/research/pu_survey/data/workbook_runs_20261025.json#w-spambase-grid/self_pu_full_meta/spambase/c0.3/seed0</t>
         </is>
       </c>
       <c r="AI25" t="inlineStr">
@@ -4184,7 +4184,7 @@
       </c>
       <c r="AH26" t="inlineStr">
         <is>
-          <t>tmp/wb_20261025/self_pu_full_meta_c0.5/ts/c_0.5/seed_0/manifest.json</t>
+          <t>docs/research/pu_survey/data/workbook_runs_20261025.json#w-spambase-grid/self_pu_full_meta/spambase/c0.5/seed0</t>
         </is>
       </c>
       <c r="AI26" t="inlineStr">
@@ -4324,7 +4324,7 @@
       </c>
       <c r="AH27" t="inlineStr">
         <is>
-          <t>tmp/wb_20261025/split_pu_c0.1/ts/c_0.1/seed_0/manifest.json</t>
+          <t>docs/research/pu_survey/data/workbook_runs_20261025.json#w-spambase-grid/split_pu/spambase/c0.1/seed0</t>
         </is>
       </c>
       <c r="AI27" t="inlineStr">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="AH28" t="inlineStr">
         <is>
-          <t>tmp/wb_20261025/split_pu_c0.3/ts/c_0.3/seed_0/manifest.json</t>
+          <t>docs/research/pu_survey/data/workbook_runs_20261025.json#w-spambase-grid/split_pu/spambase/c0.3/seed0</t>
         </is>
       </c>
       <c r="AI28" t="inlineStr">
@@ -4604,7 +4604,7 @@
       </c>
       <c r="AH29" t="inlineStr">
         <is>
-          <t>tmp/wb_20261025/split_pu_c0.5/ts/c_0.5/seed_0/manifest.json</t>
+          <t>docs/research/pu_survey/data/workbook_runs_20261025.json#w-spambase-grid/split_pu/spambase/c0.5/seed0</t>
         </is>
       </c>
       <c r="AI29" t="inlineStr">
@@ -4744,7 +4744,7 @@
       </c>
       <c r="AH30" t="inlineStr">
         <is>
-          <t>tmp/wb_20261025/upu_c0.1/ts/c_0.1/seed_0/manifest.json</t>
+          <t>docs/research/pu_survey/data/workbook_runs_20261025.json#w-spambase-grid/upu/spambase/c0.1/seed0</t>
         </is>
       </c>
       <c r="AI30" t="inlineStr">
@@ -4884,7 +4884,7 @@
       </c>
       <c r="AH31" t="inlineStr">
         <is>
-          <t>tmp/wb_20261025/upu_c0.3/ts/c_0.3/seed_0/manifest.json</t>
+          <t>docs/research/pu_survey/data/workbook_runs_20261025.json#w-spambase-grid/upu/spambase/c0.3/seed0</t>
         </is>
       </c>
       <c r="AI31" t="inlineStr">
@@ -5024,7 +5024,7 @@
       </c>
       <c r="AH32" t="inlineStr">
         <is>
-          <t>tmp/wb_20261025/upu_c0.5/ts/c_0.5/seed_0/manifest.json</t>
+          <t>docs/research/pu_survey/data/workbook_runs_20261025.json#w-spambase-grid/upu/spambase/c0.5/seed0</t>
         </is>
       </c>
       <c r="AI32" t="inlineStr">
@@ -10659,7 +10659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A50"/>
+  <dimension ref="A1:A52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="108" customWidth="1" min="1" max="1"/>
@@ -10964,14 +10964,28 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>- 工作簿：tmp/build_results_workbook_20261025.py，全部数值从 manifest 重算，不手抄。</t>
+          <t>- 工作簿：tmp/build_results_workbook_20261025.py，只读 data/workbook_runs_20261025.json，不手抄。</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>- 每行的原始 manifest 路径见 evidence_manifest 列。</t>
+          <t>- 收据：tmp/make_workbook_receipt_20261025.py 由 manifest 生成；它记录每份 manifest 的</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  sha256、被删去的 candidate_runs 轨迹摘要与 split_ref 摘要。原始 manifest 留在 tmp/，不入库。</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>- 每行的 evidence 列就是该收据里的 run key。</t>
         </is>
       </c>
     </row>

</xml_diff>